<commit_message>
Mains Board BOM with price added.
</commit_message>
<xml_diff>
--- a/Design-Files/Mains_Board/Deliverables/BOM/Client-BOM-Mains_Board.xlsx
+++ b/Design-Files/Mains_Board/Deliverables/BOM/Client-BOM-Mains_Board.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="82">
   <si>
     <t>#</t>
   </si>
@@ -234,9 +234,6 @@
     <t>Vishay</t>
   </si>
   <si>
-    <t>Comment</t>
-  </si>
-  <si>
     <t>0.1uF</t>
   </si>
   <si>
@@ -255,7 +252,19 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>#Column Name Error:' Remarks</t>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>Omron Electronics Inc-EMC Div</t>
   </si>
 </sst>
 </file>
@@ -758,9 +767,9 @@
     <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.42578125" customWidth="1"/>
+    <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -800,13 +809,13 @@
         <v>61</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="J2" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="K2" s="5" t="s">
         <v>77</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -834,7 +843,7 @@
         <v>62</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
@@ -844,7 +853,7 @@
     <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B15" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B14" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -866,7 +875,7 @@
         <v>63</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="J4" s="9">
         <v>2</v>
@@ -897,8 +906,8 @@
       <c r="H5" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="I5" s="8" t="s">
-        <v>54</v>
+      <c r="I5" s="10" t="s">
+        <v>79</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
@@ -930,7 +939,7 @@
         <v>65</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>55</v>
+        <v>79</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -952,8 +961,8 @@
       <c r="E7" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="7" t="s">
-        <v>44</v>
+      <c r="F7" s="9" t="s">
+        <v>80</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>44</v>
@@ -961,8 +970,8 @@
       <c r="H7" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I7" s="8" t="s">
-        <v>44</v>
+      <c r="I7" s="10" t="s">
+        <v>79</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -985,7 +994,7 @@
         <v>31</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>45</v>
@@ -994,7 +1003,7 @@
         <v>67</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>45</v>
+        <v>79</v>
       </c>
       <c r="J8" s="9">
         <v>3</v>
@@ -1016,13 +1025,17 @@
       <c r="E9" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="G9" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="G9" s="8"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="8" t="s">
-        <v>46</v>
+      <c r="H9" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>79</v>
       </c>
       <c r="J9" s="7">
         <v>2</v>
@@ -1054,7 +1067,7 @@
         <v>68</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="J10" s="9">
         <v>2</v>
@@ -1086,7 +1099,7 @@
         <v>69</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J11" s="7">
         <v>3</v>
@@ -1118,7 +1131,7 @@
         <v>69</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J12" s="9">
         <v>2</v>
@@ -1150,7 +1163,7 @@
         <v>69</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J13" s="7">
         <v>2</v>
@@ -1182,7 +1195,7 @@
         <v>69</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J14" s="9">
         <v>2</v>
@@ -1204,8 +1217,8 @@
       <c r="E15" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="F15" s="7" t="s">
-        <v>50</v>
+      <c r="F15" s="9" t="s">
+        <v>80</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>50</v>
@@ -1214,7 +1227,7 @@
         <v>70</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>

</xml_diff>